<commit_message>
Remove frozen panes from Excel templates to keep scrolling in one view
Keep protected examples and editable inputs while removing row/column freezing from both templates and line exports. Refresh download URLs and verify unchanged cell values, formats, protection and import/export roundtrips.
</commit_message>
<xml_diff>
--- a/assets/templates/KML_adults_template.xlsx
+++ b/assets/templates/KML_adults_template.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성충" sheetId="1" r:id="Rc5626cc4a4224c78"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="예시" sheetId="2" r:id="R7c8e161c06494bd6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="3" r:id="R67522deae4904ac1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="성충" sheetId="1" r:id="R70db85ab3699499f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="예시" sheetId="2" r:id="Re81eefcbc91a4f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="안내" sheetId="3" r:id="R4b31fdd7af714091"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>